<commit_message>
London batch 2: fix a/an and on/at wording in emails
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XgAh5ZM2DVQNBVEULsUzp1
</commit_message>
<xml_diff>
--- a/corporates/FC_Urban_London_corporates_batch2_Sep2026.xlsx
+++ b/corporates/FC_Urban_London_corporates_batch2_Sep2026.xlsx
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Third Floor, 81 Southwark Street</t>
+          <t>81 Southwark Street</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1426,7 +1426,7 @@
       <c r="T10" s="3" t="inlineStr">
         <is>
           <t>Hi Drew,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 7 minute walk from your office on Third Floor, 81 Southwark Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 7 minute walk from your office at 81 Southwark Street.
 We currently have space there on Thursdays at 20:00 and Fridays at 17:30 or 18:30.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -1512,7 +1512,7 @@
       <c r="T11" s="3" t="inlineStr">
         <is>
           <t>Hi EAM London team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 8 minute walk from your office at 215-221 Borough High Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about an 8 minute walk from your office at 215-221 Borough High Street.
 We currently have space there on Thursdays at 20:00 and Fridays at 17:30 or 18:30.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -1607,7 +1607,7 @@
         <is>
           <t>Hi Cezanne HR team,
 Congratulations on winning the 2026 Talent Tech Customer Service Award, presented in London this September.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 8 minute walk from your office at 57 Southwark Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about an 8 minute walk from your office at 57 Southwark Street.
 We currently have space there on Thursdays at 20:00 and Fridays at 17:30 or 18:30.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -1693,7 +1693,7 @@
       <c r="T13" s="3" t="inlineStr">
         <is>
           <t>Hi PensionBee team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 8 minute walk from your office at 209 Blackfriars Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about an 8 minute walk from your office at 209 Blackfriars Road.
 We currently have space there on Thursdays at 20:00 and Fridays at 17:30 or 18:30.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -2155,7 +2155,7 @@
         <is>
           <t>Hi ECD Architects team,
 Congratulations on ECD Architects making Building magazine's 2026 Top 150 Consultants list, ranking joint 36th among the Top 50 Architects.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 11 minute walk from your office at 65 Hopton Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about an 11 minute walk from your office at 65 Hopton Street.
 We currently have space there on Thursdays at 20:00 and Fridays at 17:30 or 18:30.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -2336,7 +2336,7 @@
         <is>
           <t>Hi Winckworth Sherwood team,
 Congratulations on welcoming Sean Houlihan as a new partner in the banking and finance team this September.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 12 minute walk from your office on Arbor, 255 Blackfriars Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 12 minute walk from your office at Arbor, 255 Blackfriars Road.
 We currently have space there on Thursdays at 20:00 and Fridays at 17:30 or 18:30.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -2611,7 +2611,7 @@
         <is>
           <t>Hi Hanover team,
 Congratulations on Anita Boateng joining as President in June to lead your next phase of growth.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 13 minute walk from your office on Riverside House, 2a Southwark Bridge Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 13 minute walk from your office at Riverside House, 2a Southwark Bridge Road.
 We currently have space there on Thursdays at 20:00 and Fridays at 17:30 or 18:30.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -2697,7 +2697,7 @@
       <c r="T24" s="3" t="inlineStr">
         <is>
           <t>Hi Madano team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 13 minute walk from your office on Riverside House, 2a Southwark Bridge Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 13 minute walk from your office at Riverside House, 2a Southwark Bridge Road.
 We currently have space there on Thursdays at 20:00 and Fridays at 17:30 or 18:30.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -2869,7 +2869,7 @@
       <c r="T26" s="3" t="inlineStr">
         <is>
           <t>Hi Kreab team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 15 minute walk from your office on The Shard, 32 London Bridge Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 15 minute walk from your office at The Shard, 32 London Bridge Street.
 We currently have space there on Thursdays at 20:00 and Fridays at 17:30 or 18:30.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -2955,7 +2955,7 @@
       <c r="T27" s="3" t="inlineStr">
         <is>
           <t>Hi MOBKOI team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 15 minute walk from your office on The Shard, 32 London Bridge Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy, about a 15 minute walk from your office at The Shard, 32 London Bridge Street.
 We currently have space there on Thursdays at 20:00 and Fridays at 17:30 or 18:30.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -3213,7 +3213,7 @@
       <c r="T30" s="3" t="inlineStr">
         <is>
           <t>Hi Khalij Group team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at our Poplar pitch on Poplar High Street, about a 7 minute walk from your office on One Canada Square.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at our Poplar pitch on Poplar High Street, about a 7 minute walk from your office at One Canada Square.
 We currently have space there on Tuesdays at 20:00 every week and every other Thursday at 20:00.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -3308,7 +3308,7 @@
         <is>
           <t>Hi Datatonic team,
 I saw Datatonic won two Google Cloud Partner of the Year awards this year, including UK and Ireland Country Partner.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at our Poplar pitch on Poplar High Street, about a 7 minute walk from your office on One Canada Square.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at our Poplar pitch on Poplar High Street, about a 7 minute walk from your office at One Canada Square.
 We currently have space there on Tuesdays at 20:00 every week and every other Thursday at 20:00.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -3485,7 +3485,7 @@
       <c r="T33" s="3" t="inlineStr">
         <is>
           <t>Hi Feilden+Mawson team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Coram's Fields, about a 8 minute walk from your office at 21-27 Lamb's Conduit Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Coram's Fields, about an 8 minute walk from your office at 21-27 Lamb's Conduit Street.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -3735,7 +3735,7 @@
       <c r="T36" s="3" t="inlineStr">
         <is>
           <t>Hi Insite Risk Management team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Coram's Fields, about a 11 minute walk from your office at 221 Pentonville Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Coram's Fields, about an 11 minute walk from your office at 221 Pentonville Road.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -3824,7 +3824,7 @@
       <c r="T37" s="3" t="inlineStr">
         <is>
           <t>Hi Jimmy,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Coram's Fields, about a 11 minute walk from your office at 25 Easton Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Coram's Fields, about an 11 minute walk from your office at 25 Easton Street.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -6230,7 +6230,7 @@
         <is>
           <t>Hi Essentia Analytics team,
 Congratulations on the launch of Stock Market Maestros, the book your CEO Clare Flynn Levy helped write, published this March.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Powerleague Shoreditch, about a 8 minute walk from your office at 1 Mark Square.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Powerleague Shoreditch, about an 8 minute walk from your office at 1 Mark Square.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -6309,7 +6309,7 @@
       <c r="T66" s="3" t="inlineStr">
         <is>
           <t>Hi Flexciton team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Powerleague Shoreditch, about a 8 minute walk from your office on Curtain Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Powerleague Shoreditch, about an 8 minute walk from your office on Curtain Road.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -6804,7 +6804,7 @@
       <c r="T72" s="3" t="inlineStr">
         <is>
           <t>Hi Rosco team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Rosemary Gardens in Islington, about a 8 minute walk from your office on De Beauvoir Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Rosemary Gardens in Islington, about an 8 minute walk from your office on De Beauvoir Road.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -7226,7 +7226,7 @@
       <c r="T77" s="3" t="inlineStr">
         <is>
           <t>Hi Gemic team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at our South Kensington pitch on Thomas More Walk, about a 2 minute walk from your office on Michelin House, 81 Fulham Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at our South Kensington pitch on Thomas More Walk, about a 2 minute walk from your office at Michelin House, 81 Fulham Road.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -7577,7 +7577,7 @@
       <c r="T81" s="3" t="inlineStr">
         <is>
           <t>Hi Kefron team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at our South Kensington pitch on Thomas More Walk, about a 11 minute walk from your office at 21 Ellis Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at our South Kensington pitch on Thomas More Walk, about an 11 minute walk from your office at 21 Ellis Street.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -7658,7 +7658,7 @@
       <c r="T82" s="3" t="inlineStr">
         <is>
           <t>Hi venturethree team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at our South Kensington pitch on Thomas More Walk, about a 11 minute walk from your office at 11 Cavalry Square.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at our South Kensington pitch on Thomas More Walk, about an 11 minute walk from your office at 11 Cavalry Square.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -8679,7 +8679,7 @@
       <c r="T94" s="3" t="inlineStr">
         <is>
           <t>Hi DVF Recruitment team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at the Attlee Centre on Thrawl Street, about a 8 minute walk from your office at 10-12 Alie Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at the Attlee Centre on Thrawl Street, about an 8 minute walk from your office at 10-12 Alie Street.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -8939,7 +8939,7 @@
         <is>
           <t>Hi Northell team,
 Congratulations on your December 2025 partnership with Clearcast, bringing Northell's explainable AI to UK television ad clearance.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at the Attlee Centre on Thrawl Street, about a 10 minute walk from your office on Heron Tower, 110 Bishopsgate.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at the Attlee Centre on Thrawl Street, about a 10 minute walk from your office at Heron Tower, 110 Bishopsgate.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -9049,7 +9049,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>18th Floor, 100 Bishopsgate</t>
+          <t>100 Bishopsgate</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -9099,7 +9099,7 @@
       <c r="T99" s="3" t="inlineStr">
         <is>
           <t>Hi Celon team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at the Attlee Centre on Thrawl Street, about a 10 minute walk from your office at 18th Floor, 100 Bishopsgate.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at the Attlee Centre on Thrawl Street, about a 10 minute walk from your office at 100 Bishopsgate.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -9287,7 +9287,7 @@
         <is>
           <t>Hi Two Three Bird team,
 I saw your Sundays brand launched new electric bike insurance cover for UK delivery riders this January.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at the Attlee Centre on Thrawl Street, about a 11 minute walk from your office at 5 St Helen's Place.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at the Attlee Centre on Thrawl Street, about an 11 minute walk from your office at 5 St Helen's Place.
 We'd love to help start a regular after work game for the team. We handle the pitch, the organisation and the payments, and if a few people can't make it we fill the spare places with our own players.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,

</xml_diff>